<commit_message>
Add overall-market composite chart
Equal-weight, chain-linked geometric-mean composite of the 10 games'
median fixed-basket indices (all products, singles, sealed), with
individual game lines as context; appends a Market composite sheet
to the workbook.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GzVZ7jTqTdEEWEf8Dpoz9q
</commit_message>
<xml_diff>
--- a/output/tcg_price_trends.xlsx
+++ b/output/tcg_price_trends.xlsx
@@ -19,6 +19,7 @@
     <sheet name="Digimon" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="DBS Fusion World" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="Weiss Schwarz" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Market composite" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -570,8 +571,6 @@
       <c r="K2" t="n">
         <v>100</v>
       </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
       <c r="N2" t="n">
         <v>100</v>
       </c>
@@ -584,8 +583,6 @@
       <c r="Q2" t="n">
         <v>100</v>
       </c>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
       <c r="T2" t="n">
         <v>100</v>
       </c>
@@ -629,8 +626,6 @@
       <c r="K3" t="n">
         <v>94.16767257388445</v>
       </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
       <c r="N3" t="n">
         <v>100</v>
       </c>
@@ -5479,6 +5474,522 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>market_composite</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>singles_composite</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>sealed_composite</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2024-02</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>100</v>
+      </c>
+      <c r="C2" t="n">
+        <v>100</v>
+      </c>
+      <c r="D2" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2024-03</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>100</v>
+      </c>
+      <c r="C3" t="n">
+        <v>100</v>
+      </c>
+      <c r="D3" t="n">
+        <v>99.12279261508665</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2024-04</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>93.53502782715402</v>
+      </c>
+      <c r="C4" t="n">
+        <v>93.48245267654265</v>
+      </c>
+      <c r="D4" t="n">
+        <v>95.43990211401469</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2024-05</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>91.41235653250047</v>
+      </c>
+      <c r="C5" t="n">
+        <v>91.33533223327724</v>
+      </c>
+      <c r="D5" t="n">
+        <v>100.7982532269792</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2024-06</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>88.2706452826597</v>
+      </c>
+      <c r="C6" t="n">
+        <v>88.05346980368091</v>
+      </c>
+      <c r="D6" t="n">
+        <v>96.95747821054657</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2024-07</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>85.46626320032829</v>
+      </c>
+      <c r="C7" t="n">
+        <v>85.27501142820051</v>
+      </c>
+      <c r="D7" t="n">
+        <v>91.08663593451932</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2024-08</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>83.28206977248065</v>
+      </c>
+      <c r="C8" t="n">
+        <v>83.18824157362505</v>
+      </c>
+      <c r="D8" t="n">
+        <v>88.34627008478817</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2024-09</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>82.31345912458332</v>
+      </c>
+      <c r="C9" t="n">
+        <v>82.18852060229668</v>
+      </c>
+      <c r="D9" t="n">
+        <v>88.19508259565525</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2024-10</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>81.42278512366728</v>
+      </c>
+      <c r="C10" t="n">
+        <v>81.34607525454577</v>
+      </c>
+      <c r="D10" t="n">
+        <v>86.86802145574863</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2024-11</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>80.11295607442578</v>
+      </c>
+      <c r="C11" t="n">
+        <v>80.02187866361527</v>
+      </c>
+      <c r="D11" t="n">
+        <v>86.6873118302408</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2024-12</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>79.64468877265514</v>
+      </c>
+      <c r="C12" t="n">
+        <v>79.53472902230985</v>
+      </c>
+      <c r="D12" t="n">
+        <v>84.8926954687828</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>79.35830128820649</v>
+      </c>
+      <c r="C13" t="n">
+        <v>79.22423874868635</v>
+      </c>
+      <c r="D13" t="n">
+        <v>85.3004823258386</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2025-02</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>79.47198882375508</v>
+      </c>
+      <c r="C14" t="n">
+        <v>79.25036777818175</v>
+      </c>
+      <c r="D14" t="n">
+        <v>84.79366898122588</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>80.45455045837473</v>
+      </c>
+      <c r="C15" t="n">
+        <v>80.14651141368498</v>
+      </c>
+      <c r="D15" t="n">
+        <v>85.99658806784304</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2025-04</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>80.76079388011331</v>
+      </c>
+      <c r="C16" t="n">
+        <v>80.45665322473684</v>
+      </c>
+      <c r="D16" t="n">
+        <v>87.77999384958204</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2025-05</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>80.48912979459143</v>
+      </c>
+      <c r="C17" t="n">
+        <v>80.07798632318567</v>
+      </c>
+      <c r="D17" t="n">
+        <v>87.45912188156673</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>80.02803907169742</v>
+      </c>
+      <c r="C18" t="n">
+        <v>79.65852121145002</v>
+      </c>
+      <c r="D18" t="n">
+        <v>88.06241123607917</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2025-07</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>80.09692437944288</v>
+      </c>
+      <c r="C19" t="n">
+        <v>79.78497691278277</v>
+      </c>
+      <c r="D19" t="n">
+        <v>91.41741638953266</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2025-08</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>80.56645016566674</v>
+      </c>
+      <c r="C20" t="n">
+        <v>80.19723663348906</v>
+      </c>
+      <c r="D20" t="n">
+        <v>92.61817326363897</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2025-09</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>80.18505043308154</v>
+      </c>
+      <c r="C21" t="n">
+        <v>79.73729087283778</v>
+      </c>
+      <c r="D21" t="n">
+        <v>92.84839388114507</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>80.87829694276101</v>
+      </c>
+      <c r="C22" t="n">
+        <v>80.16889294899508</v>
+      </c>
+      <c r="D22" t="n">
+        <v>95.49276188060566</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2025-11</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>80.36936099535117</v>
+      </c>
+      <c r="C23" t="n">
+        <v>79.88541611841178</v>
+      </c>
+      <c r="D23" t="n">
+        <v>97.06605925502149</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>79.75399579151699</v>
+      </c>
+      <c r="C24" t="n">
+        <v>79.31361451956276</v>
+      </c>
+      <c r="D24" t="n">
+        <v>98.53561074550082</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>80.37680999091492</v>
+      </c>
+      <c r="C25" t="n">
+        <v>79.83803673999617</v>
+      </c>
+      <c r="D25" t="n">
+        <v>100.1882404553362</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>81.18090769527777</v>
+      </c>
+      <c r="C26" t="n">
+        <v>80.67111449675924</v>
+      </c>
+      <c r="D26" t="n">
+        <v>103.1382392514146</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>82.82088037488425</v>
+      </c>
+      <c r="C27" t="n">
+        <v>82.33642675035576</v>
+      </c>
+      <c r="D27" t="n">
+        <v>103.0364367180556</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>83.94164904105426</v>
+      </c>
+      <c r="C28" t="n">
+        <v>83.50627718044846</v>
+      </c>
+      <c r="D28" t="n">
+        <v>102.8019087193787</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>85.60926267760219</v>
+      </c>
+      <c r="C29" t="n">
+        <v>85.08031850976975</v>
+      </c>
+      <c r="D29" t="n">
+        <v>104.8742151208527</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>86.06372611542771</v>
+      </c>
+      <c r="C30" t="n">
+        <v>85.6527429808706</v>
+      </c>
+      <c r="D30" t="n">
+        <v>105.9532239252203</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>87.69557738496161</v>
+      </c>
+      <c r="C31" t="n">
+        <v>86.7872175133388</v>
+      </c>
+      <c r="D31" t="n">
+        <v>106.1723537051054</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Switch market composite to value weighting
Headline series is now the chained aggregate market value of the fixed
baskets (games weighted by basket value: Magic 50%, Pokemon 21%,
Yu-Gi-Oh 17% at base), a cap-weighted-style market proxy. Equal-weight
median kept as a dashed 'typical game' reference.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GzVZ7jTqTdEEWEf8Dpoz9q
</commit_message>
<xml_diff>
--- a/output/tcg_price_trends.xlsx
+++ b/output/tcg_price_trends.xlsx
@@ -5480,7 +5480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5491,17 +5491,22 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>market_composite</t>
+          <t>market_value_weighted</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>singles_composite</t>
+          <t>singles_value_weighted</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>sealed_composite</t>
+          <t>sealed_value_weighted</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>equal_weight_typical_game</t>
         </is>
       </c>
     </row>
@@ -5520,6 +5525,9 @@
       <c r="D2" t="n">
         <v>100</v>
       </c>
+      <c r="E2" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -5528,13 +5536,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>100</v>
+        <v>99.4249880578468</v>
       </c>
       <c r="C3" t="n">
-        <v>100</v>
+        <v>99.26796824752843</v>
       </c>
       <c r="D3" t="n">
-        <v>99.12279261508665</v>
+        <v>100.1020089845326</v>
+      </c>
+      <c r="E3" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="4">
@@ -5544,13 +5555,16 @@
         </is>
       </c>
       <c r="B4" t="n">
+        <v>99.41613325521311</v>
+      </c>
+      <c r="C4" t="n">
+        <v>99.03006907207417</v>
+      </c>
+      <c r="D4" t="n">
+        <v>101.0740959740587</v>
+      </c>
+      <c r="E4" t="n">
         <v>93.53502782715402</v>
-      </c>
-      <c r="C4" t="n">
-        <v>93.48245267654265</v>
-      </c>
-      <c r="D4" t="n">
-        <v>95.43990211401469</v>
       </c>
     </row>
     <row r="5">
@@ -5560,13 +5574,16 @@
         </is>
       </c>
       <c r="B5" t="n">
+        <v>100.2615529233542</v>
+      </c>
+      <c r="C5" t="n">
+        <v>99.80339495829791</v>
+      </c>
+      <c r="D5" t="n">
+        <v>102.2296558037949</v>
+      </c>
+      <c r="E5" t="n">
         <v>91.41235653250047</v>
-      </c>
-      <c r="C5" t="n">
-        <v>91.33533223327724</v>
-      </c>
-      <c r="D5" t="n">
-        <v>100.7982532269792</v>
       </c>
     </row>
     <row r="6">
@@ -5576,13 +5593,16 @@
         </is>
       </c>
       <c r="B6" t="n">
+        <v>100.115941689109</v>
+      </c>
+      <c r="C6" t="n">
+        <v>99.30512330335259</v>
+      </c>
+      <c r="D6" t="n">
+        <v>103.6012824685546</v>
+      </c>
+      <c r="E6" t="n">
         <v>88.2706452826597</v>
-      </c>
-      <c r="C6" t="n">
-        <v>88.05346980368091</v>
-      </c>
-      <c r="D6" t="n">
-        <v>96.95747821054657</v>
       </c>
     </row>
     <row r="7">
@@ -5592,13 +5612,16 @@
         </is>
       </c>
       <c r="B7" t="n">
+        <v>100.0828826306187</v>
+      </c>
+      <c r="C7" t="n">
+        <v>99.1871279332664</v>
+      </c>
+      <c r="D7" t="n">
+        <v>103.9336417051764</v>
+      </c>
+      <c r="E7" t="n">
         <v>85.46626320032829</v>
-      </c>
-      <c r="C7" t="n">
-        <v>85.27501142820051</v>
-      </c>
-      <c r="D7" t="n">
-        <v>91.08663593451932</v>
       </c>
     </row>
     <row r="8">
@@ -5608,13 +5631,16 @@
         </is>
       </c>
       <c r="B8" t="n">
+        <v>99.28602085417771</v>
+      </c>
+      <c r="C8" t="n">
+        <v>98.27076440431765</v>
+      </c>
+      <c r="D8" t="n">
+        <v>103.6509303268448</v>
+      </c>
+      <c r="E8" t="n">
         <v>83.28206977248065</v>
-      </c>
-      <c r="C8" t="n">
-        <v>83.18824157362505</v>
-      </c>
-      <c r="D8" t="n">
-        <v>88.34627008478817</v>
       </c>
     </row>
     <row r="9">
@@ -5624,13 +5650,16 @@
         </is>
       </c>
       <c r="B9" t="n">
+        <v>99.48017816698972</v>
+      </c>
+      <c r="C9" t="n">
+        <v>98.31097908498552</v>
+      </c>
+      <c r="D9" t="n">
+        <v>104.5073816077857</v>
+      </c>
+      <c r="E9" t="n">
         <v>82.31345912458332</v>
-      </c>
-      <c r="C9" t="n">
-        <v>82.18852060229668</v>
-      </c>
-      <c r="D9" t="n">
-        <v>88.19508259565525</v>
       </c>
     </row>
     <row r="10">
@@ -5640,13 +5669,16 @@
         </is>
       </c>
       <c r="B10" t="n">
+        <v>99.00110913119971</v>
+      </c>
+      <c r="C10" t="n">
+        <v>97.41051798671734</v>
+      </c>
+      <c r="D10" t="n">
+        <v>105.8412612255604</v>
+      </c>
+      <c r="E10" t="n">
         <v>81.42278512366728</v>
-      </c>
-      <c r="C10" t="n">
-        <v>81.34607525454577</v>
-      </c>
-      <c r="D10" t="n">
-        <v>86.86802145574863</v>
       </c>
     </row>
     <row r="11">
@@ -5656,13 +5688,16 @@
         </is>
       </c>
       <c r="B11" t="n">
+        <v>98.88524421484993</v>
+      </c>
+      <c r="C11" t="n">
+        <v>96.81299964875683</v>
+      </c>
+      <c r="D11" t="n">
+        <v>107.7975935404891</v>
+      </c>
+      <c r="E11" t="n">
         <v>80.11295607442578</v>
-      </c>
-      <c r="C11" t="n">
-        <v>80.02187866361527</v>
-      </c>
-      <c r="D11" t="n">
-        <v>86.6873118302408</v>
       </c>
     </row>
     <row r="12">
@@ -5672,13 +5707,16 @@
         </is>
       </c>
       <c r="B12" t="n">
+        <v>98.83509323750631</v>
+      </c>
+      <c r="C12" t="n">
+        <v>96.22191112565937</v>
+      </c>
+      <c r="D12" t="n">
+        <v>110.0746929859902</v>
+      </c>
+      <c r="E12" t="n">
         <v>79.64468877265514</v>
-      </c>
-      <c r="C12" t="n">
-        <v>79.53472902230985</v>
-      </c>
-      <c r="D12" t="n">
-        <v>84.8926954687828</v>
       </c>
     </row>
     <row r="13">
@@ -5688,13 +5726,16 @@
         </is>
       </c>
       <c r="B13" t="n">
+        <v>100.2478842822831</v>
+      </c>
+      <c r="C13" t="n">
+        <v>97.12943326920076</v>
+      </c>
+      <c r="D13" t="n">
+        <v>113.6612351201878</v>
+      </c>
+      <c r="E13" t="n">
         <v>79.35830128820649</v>
-      </c>
-      <c r="C13" t="n">
-        <v>79.22423874868635</v>
-      </c>
-      <c r="D13" t="n">
-        <v>85.3004823258386</v>
       </c>
     </row>
     <row r="14">
@@ -5704,13 +5745,16 @@
         </is>
       </c>
       <c r="B14" t="n">
+        <v>102.1353794094423</v>
+      </c>
+      <c r="C14" t="n">
+        <v>98.18865349508739</v>
+      </c>
+      <c r="D14" t="n">
+        <v>119.112119877118</v>
+      </c>
+      <c r="E14" t="n">
         <v>79.47198882375508</v>
-      </c>
-      <c r="C14" t="n">
-        <v>79.25036777818175</v>
-      </c>
-      <c r="D14" t="n">
-        <v>84.79366898122588</v>
       </c>
     </row>
     <row r="15">
@@ -5720,13 +5764,16 @@
         </is>
       </c>
       <c r="B15" t="n">
+        <v>104.4251674761928</v>
+      </c>
+      <c r="C15" t="n">
+        <v>100.1313196759813</v>
+      </c>
+      <c r="D15" t="n">
+        <v>122.8952446233194</v>
+      </c>
+      <c r="E15" t="n">
         <v>80.45455045837473</v>
-      </c>
-      <c r="C15" t="n">
-        <v>80.14651141368498</v>
-      </c>
-      <c r="D15" t="n">
-        <v>85.99658806784304</v>
       </c>
     </row>
     <row r="16">
@@ -5736,13 +5783,16 @@
         </is>
       </c>
       <c r="B16" t="n">
+        <v>107.4640104055557</v>
+      </c>
+      <c r="C16" t="n">
+        <v>102.5681259164049</v>
+      </c>
+      <c r="D16" t="n">
+        <v>128.5241091451082</v>
+      </c>
+      <c r="E16" t="n">
         <v>80.76079388011331</v>
-      </c>
-      <c r="C16" t="n">
-        <v>80.45665322473684</v>
-      </c>
-      <c r="D16" t="n">
-        <v>87.77999384958204</v>
       </c>
     </row>
     <row r="17">
@@ -5752,13 +5802,16 @@
         </is>
       </c>
       <c r="B17" t="n">
+        <v>109.4193137718079</v>
+      </c>
+      <c r="C17" t="n">
+        <v>104.0017749665367</v>
+      </c>
+      <c r="D17" t="n">
+        <v>132.7236414892755</v>
+      </c>
+      <c r="E17" t="n">
         <v>80.48912979459143</v>
-      </c>
-      <c r="C17" t="n">
-        <v>80.07798632318567</v>
-      </c>
-      <c r="D17" t="n">
-        <v>87.45912188156673</v>
       </c>
     </row>
     <row r="18">
@@ -5768,13 +5821,16 @@
         </is>
       </c>
       <c r="B18" t="n">
+        <v>112.0314434800046</v>
+      </c>
+      <c r="C18" t="n">
+        <v>105.3744088901189</v>
+      </c>
+      <c r="D18" t="n">
+        <v>140.668314411231</v>
+      </c>
+      <c r="E18" t="n">
         <v>80.02803907169742</v>
-      </c>
-      <c r="C18" t="n">
-        <v>79.65852121145002</v>
-      </c>
-      <c r="D18" t="n">
-        <v>88.06241123607917</v>
       </c>
     </row>
     <row r="19">
@@ -5784,13 +5840,16 @@
         </is>
       </c>
       <c r="B19" t="n">
+        <v>113.3302723669756</v>
+      </c>
+      <c r="C19" t="n">
+        <v>105.4536756227929</v>
+      </c>
+      <c r="D19" t="n">
+        <v>147.2139664324793</v>
+      </c>
+      <c r="E19" t="n">
         <v>80.09692437944288</v>
-      </c>
-      <c r="C19" t="n">
-        <v>79.78497691278277</v>
-      </c>
-      <c r="D19" t="n">
-        <v>91.41741638953266</v>
       </c>
     </row>
     <row r="20">
@@ -5800,13 +5859,16 @@
         </is>
       </c>
       <c r="B20" t="n">
+        <v>116.7187081527943</v>
+      </c>
+      <c r="C20" t="n">
+        <v>107.6653416306083</v>
+      </c>
+      <c r="D20" t="n">
+        <v>155.6650591413649</v>
+      </c>
+      <c r="E20" t="n">
         <v>80.56645016566674</v>
-      </c>
-      <c r="C20" t="n">
-        <v>80.19723663348906</v>
-      </c>
-      <c r="D20" t="n">
-        <v>92.61817326363897</v>
       </c>
     </row>
     <row r="21">
@@ -5816,13 +5878,16 @@
         </is>
       </c>
       <c r="B21" t="n">
+        <v>120.2682573812531</v>
+      </c>
+      <c r="C21" t="n">
+        <v>109.4265347883264</v>
+      </c>
+      <c r="D21" t="n">
+        <v>166.9084579974951</v>
+      </c>
+      <c r="E21" t="n">
         <v>80.18505043308154</v>
-      </c>
-      <c r="C21" t="n">
-        <v>79.73729087283778</v>
-      </c>
-      <c r="D21" t="n">
-        <v>92.84839388114507</v>
       </c>
     </row>
     <row r="22">
@@ -5832,13 +5897,16 @@
         </is>
       </c>
       <c r="B22" t="n">
+        <v>123.7727403432192</v>
+      </c>
+      <c r="C22" t="n">
+        <v>111.7679784405948</v>
+      </c>
+      <c r="D22" t="n">
+        <v>175.4165224850115</v>
+      </c>
+      <c r="E22" t="n">
         <v>80.87829694276101</v>
-      </c>
-      <c r="C22" t="n">
-        <v>80.16889294899508</v>
-      </c>
-      <c r="D22" t="n">
-        <v>95.49276188060566</v>
       </c>
     </row>
     <row r="23">
@@ -5848,13 +5916,16 @@
         </is>
       </c>
       <c r="B23" t="n">
+        <v>125.9604949871992</v>
+      </c>
+      <c r="C23" t="n">
+        <v>113.1334317282987</v>
+      </c>
+      <c r="D23" t="n">
+        <v>181.1419580639499</v>
+      </c>
+      <c r="E23" t="n">
         <v>80.36936099535117</v>
-      </c>
-      <c r="C23" t="n">
-        <v>79.88541611841178</v>
-      </c>
-      <c r="D23" t="n">
-        <v>97.06605925502149</v>
       </c>
     </row>
     <row r="24">
@@ -5864,13 +5935,16 @@
         </is>
       </c>
       <c r="B24" t="n">
+        <v>128.097291141673</v>
+      </c>
+      <c r="C24" t="n">
+        <v>114.1725919301347</v>
+      </c>
+      <c r="D24" t="n">
+        <v>188.0009951335699</v>
+      </c>
+      <c r="E24" t="n">
         <v>79.75399579151699</v>
-      </c>
-      <c r="C24" t="n">
-        <v>79.31361451956276</v>
-      </c>
-      <c r="D24" t="n">
-        <v>98.53561074550082</v>
       </c>
     </row>
     <row r="25">
@@ -5880,13 +5954,16 @@
         </is>
       </c>
       <c r="B25" t="n">
+        <v>131.4440662190809</v>
+      </c>
+      <c r="C25" t="n">
+        <v>116.8349325322026</v>
+      </c>
+      <c r="D25" t="n">
+        <v>194.2922784981469</v>
+      </c>
+      <c r="E25" t="n">
         <v>80.37680999091492</v>
-      </c>
-      <c r="C25" t="n">
-        <v>79.83803673999617</v>
-      </c>
-      <c r="D25" t="n">
-        <v>100.1882404553362</v>
       </c>
     </row>
     <row r="26">
@@ -5896,13 +5973,16 @@
         </is>
       </c>
       <c r="B26" t="n">
+        <v>136.1309773416151</v>
+      </c>
+      <c r="C26" t="n">
+        <v>119.8466399274315</v>
+      </c>
+      <c r="D26" t="n">
+        <v>206.1861953857602</v>
+      </c>
+      <c r="E26" t="n">
         <v>81.18090769527777</v>
-      </c>
-      <c r="C26" t="n">
-        <v>80.67111449675924</v>
-      </c>
-      <c r="D26" t="n">
-        <v>103.1382392514146</v>
       </c>
     </row>
     <row r="27">
@@ -5912,13 +5992,16 @@
         </is>
       </c>
       <c r="B27" t="n">
+        <v>140.0609263952016</v>
+      </c>
+      <c r="C27" t="n">
+        <v>123.6570430557842</v>
+      </c>
+      <c r="D27" t="n">
+        <v>210.6303430901159</v>
+      </c>
+      <c r="E27" t="n">
         <v>82.82088037488425</v>
-      </c>
-      <c r="C27" t="n">
-        <v>82.33642675035576</v>
-      </c>
-      <c r="D27" t="n">
-        <v>103.0364367180556</v>
       </c>
     </row>
     <row r="28">
@@ -5928,13 +6011,16 @@
         </is>
       </c>
       <c r="B28" t="n">
+        <v>144.9088277662518</v>
+      </c>
+      <c r="C28" t="n">
+        <v>127.8754331719986</v>
+      </c>
+      <c r="D28" t="n">
+        <v>218.1864142570606</v>
+      </c>
+      <c r="E28" t="n">
         <v>83.94164904105426</v>
-      </c>
-      <c r="C28" t="n">
-        <v>83.50627718044846</v>
-      </c>
-      <c r="D28" t="n">
-        <v>102.8019087193787</v>
       </c>
     </row>
     <row r="29">
@@ -5944,13 +6030,16 @@
         </is>
       </c>
       <c r="B29" t="n">
+        <v>149.7006471223579</v>
+      </c>
+      <c r="C29" t="n">
+        <v>132.5301178921778</v>
+      </c>
+      <c r="D29" t="n">
+        <v>223.5680774528964</v>
+      </c>
+      <c r="E29" t="n">
         <v>85.60926267760219</v>
-      </c>
-      <c r="C29" t="n">
-        <v>85.08031850976975</v>
-      </c>
-      <c r="D29" t="n">
-        <v>104.8742151208527</v>
       </c>
     </row>
     <row r="30">
@@ -5960,13 +6049,16 @@
         </is>
       </c>
       <c r="B30" t="n">
+        <v>157.3558598819894</v>
+      </c>
+      <c r="C30" t="n">
+        <v>138.9963995702695</v>
+      </c>
+      <c r="D30" t="n">
+        <v>236.3381401219637</v>
+      </c>
+      <c r="E30" t="n">
         <v>86.06372611542771</v>
-      </c>
-      <c r="C30" t="n">
-        <v>85.6527429808706</v>
-      </c>
-      <c r="D30" t="n">
-        <v>105.9532239252203</v>
       </c>
     </row>
     <row r="31">
@@ -5976,13 +6068,16 @@
         </is>
       </c>
       <c r="B31" t="n">
+        <v>164.1425431061003</v>
+      </c>
+      <c r="C31" t="n">
+        <v>145.161794406534</v>
+      </c>
+      <c r="D31" t="n">
+        <v>245.7975581495947</v>
+      </c>
+      <c r="E31" t="n">
         <v>87.69557738496161</v>
-      </c>
-      <c r="C31" t="n">
-        <v>86.7872175133388</v>
-      </c>
-      <c r="D31" t="n">
-        <v>106.1723537051054</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Weight market composite by realized TCGplayer GMV
Cross-game weights now come from a client-provided 3-month realized
GMV summary (Magic 40%, Pokemon 32%, One Piece 13% of top-10 total)
instead of basket value; weights stored in tcg_config.GMV_3MO.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GzVZ7jTqTdEEWEf8Dpoz9q
</commit_message>
<xml_diff>
--- a/output/tcg_price_trends.xlsx
+++ b/output/tcg_price_trends.xlsx
@@ -5491,17 +5491,17 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>market_value_weighted</t>
+          <t>market_gmv_weighted</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>singles_value_weighted</t>
+          <t>singles_gmv_weighted</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>sealed_value_weighted</t>
+          <t>sealed_gmv_weighted</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
@@ -5536,13 +5536,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>99.4249880578468</v>
+        <v>99.17898266003334</v>
       </c>
       <c r="C3" t="n">
-        <v>99.26796824752843</v>
+        <v>98.70207950425358</v>
       </c>
       <c r="D3" t="n">
-        <v>100.1020089845326</v>
+        <v>100.0488886357012</v>
       </c>
       <c r="E3" t="n">
         <v>100</v>
@@ -5555,13 +5555,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>99.41613325521311</v>
+        <v>99.14277566706055</v>
       </c>
       <c r="C4" t="n">
-        <v>99.03006907207417</v>
+        <v>97.84880194052732</v>
       </c>
       <c r="D4" t="n">
-        <v>101.0740959740587</v>
+        <v>101.4141811287269</v>
       </c>
       <c r="E4" t="n">
         <v>93.53502782715402</v>
@@ -5574,13 +5574,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>100.2615529233542</v>
+        <v>100.2476838600313</v>
       </c>
       <c r="C5" t="n">
-        <v>99.80339495829791</v>
+        <v>98.99319912552043</v>
       </c>
       <c r="D5" t="n">
-        <v>102.2296558037949</v>
+        <v>102.5003015605024</v>
       </c>
       <c r="E5" t="n">
         <v>91.41235653250047</v>
@@ -5593,13 +5593,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>100.115941689109</v>
+        <v>99.95212691020669</v>
       </c>
       <c r="C6" t="n">
-        <v>99.30512330335259</v>
+        <v>98.33690206012628</v>
       </c>
       <c r="D6" t="n">
-        <v>103.6012824685546</v>
+        <v>103.5785189610995</v>
       </c>
       <c r="E6" t="n">
         <v>88.2706452826597</v>
@@ -5612,13 +5612,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>100.0828826306187</v>
+        <v>99.15295469964164</v>
       </c>
       <c r="C7" t="n">
-        <v>99.1871279332664</v>
+        <v>97.45121315695368</v>
       </c>
       <c r="D7" t="n">
-        <v>103.9336417051764</v>
+        <v>103.2581444320212</v>
       </c>
       <c r="E7" t="n">
         <v>85.46626320032829</v>
@@ -5631,13 +5631,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>99.28602085417771</v>
+        <v>96.63767113211858</v>
       </c>
       <c r="C8" t="n">
-        <v>98.27076440431765</v>
+        <v>94.84287490257303</v>
       </c>
       <c r="D8" t="n">
-        <v>103.6509303268448</v>
+        <v>101.5192274928585</v>
       </c>
       <c r="E8" t="n">
         <v>83.28206977248065</v>
@@ -5650,13 +5650,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>99.48017816698972</v>
+        <v>96.06737373749505</v>
       </c>
       <c r="C9" t="n">
-        <v>98.31097908498552</v>
+        <v>94.12064908734558</v>
       </c>
       <c r="D9" t="n">
-        <v>104.5073816077857</v>
+        <v>101.5284704716153</v>
       </c>
       <c r="E9" t="n">
         <v>82.31345912458332</v>
@@ -5669,13 +5669,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>99.00110913119971</v>
+        <v>95.45881350338993</v>
       </c>
       <c r="C10" t="n">
-        <v>97.41051798671734</v>
+        <v>92.57702683055211</v>
       </c>
       <c r="D10" t="n">
-        <v>105.8412612255604</v>
+        <v>103.1115175311061</v>
       </c>
       <c r="E10" t="n">
         <v>81.42278512366728</v>
@@ -5688,13 +5688,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>98.88524421484993</v>
+        <v>95.53422284930724</v>
       </c>
       <c r="C11" t="n">
-        <v>96.81299964875683</v>
+        <v>91.86137987731917</v>
       </c>
       <c r="D11" t="n">
-        <v>107.7975935404891</v>
+        <v>105.2246770728277</v>
       </c>
       <c r="E11" t="n">
         <v>80.11295607442578</v>
@@ -5707,13 +5707,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>98.83509323750631</v>
+        <v>95.70855682283199</v>
       </c>
       <c r="C12" t="n">
-        <v>96.22191112565937</v>
+        <v>91.30110048598537</v>
       </c>
       <c r="D12" t="n">
-        <v>110.0746929859902</v>
+        <v>107.302433662846</v>
       </c>
       <c r="E12" t="n">
         <v>79.64468877265514</v>
@@ -5726,13 +5726,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>100.2478842822831</v>
+        <v>97.19577771802645</v>
       </c>
       <c r="C13" t="n">
-        <v>97.12943326920076</v>
+        <v>92.2491018473451</v>
       </c>
       <c r="D13" t="n">
-        <v>113.6612351201878</v>
+        <v>110.2127973509421</v>
       </c>
       <c r="E13" t="n">
         <v>79.35830128820649</v>
@@ -5745,13 +5745,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>102.1353794094423</v>
+        <v>99.92110855098751</v>
       </c>
       <c r="C14" t="n">
-        <v>98.18865349508739</v>
+        <v>94.18397213281668</v>
       </c>
       <c r="D14" t="n">
-        <v>119.112119877118</v>
+        <v>115.3776845748422</v>
       </c>
       <c r="E14" t="n">
         <v>79.47198882375508</v>
@@ -5764,13 +5764,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>104.4251674761928</v>
+        <v>102.6860083351276</v>
       </c>
       <c r="C15" t="n">
-        <v>100.1313196759813</v>
+        <v>96.69980778909682</v>
       </c>
       <c r="D15" t="n">
-        <v>122.8952446233194</v>
+        <v>118.8852537274126</v>
       </c>
       <c r="E15" t="n">
         <v>80.45455045837473</v>
@@ -5783,13 +5783,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>107.4640104055557</v>
+        <v>105.935540695292</v>
       </c>
       <c r="C16" t="n">
-        <v>102.5681259164049</v>
+        <v>99.07305804694079</v>
       </c>
       <c r="D16" t="n">
-        <v>128.5241091451082</v>
+        <v>124.0273208805642</v>
       </c>
       <c r="E16" t="n">
         <v>80.76079388011331</v>
@@ -5802,13 +5802,13 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>109.4193137718079</v>
+        <v>107.8433416342542</v>
       </c>
       <c r="C17" t="n">
-        <v>104.0017749665367</v>
+        <v>100.0099937294076</v>
       </c>
       <c r="D17" t="n">
-        <v>132.7236414892755</v>
+        <v>127.8306068026426</v>
       </c>
       <c r="E17" t="n">
         <v>80.48912979459143</v>
@@ -5821,13 +5821,13 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>112.0314434800046</v>
+        <v>110.4328483943508</v>
       </c>
       <c r="C18" t="n">
-        <v>105.3744088901189</v>
+        <v>100.7370822893562</v>
       </c>
       <c r="D18" t="n">
-        <v>140.668314411231</v>
+        <v>134.604204813265</v>
       </c>
       <c r="E18" t="n">
         <v>80.02803907169742</v>
@@ -5840,13 +5840,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>113.3302723669756</v>
+        <v>111.6546956959033</v>
       </c>
       <c r="C19" t="n">
-        <v>105.4536756227929</v>
+        <v>100.4326484261568</v>
       </c>
       <c r="D19" t="n">
-        <v>147.2139664324793</v>
+        <v>140.0069680458598</v>
       </c>
       <c r="E19" t="n">
         <v>80.09692437944288</v>
@@ -5859,13 +5859,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>116.7187081527943</v>
+        <v>114.947705285885</v>
       </c>
       <c r="C20" t="n">
-        <v>107.6653416306083</v>
+        <v>102.4631339555483</v>
       </c>
       <c r="D20" t="n">
-        <v>155.6650591413649</v>
+        <v>146.4992698784768</v>
       </c>
       <c r="E20" t="n">
         <v>80.56645016566674</v>
@@ -5878,13 +5878,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>120.2682573812531</v>
+        <v>118.6016626047306</v>
       </c>
       <c r="C21" t="n">
-        <v>109.4265347883264</v>
+        <v>104.1817141371515</v>
       </c>
       <c r="D21" t="n">
-        <v>166.9084579974951</v>
+        <v>155.1634280914048</v>
       </c>
       <c r="E21" t="n">
         <v>80.18505043308154</v>
@@ -5897,13 +5897,13 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>123.7727403432192</v>
+        <v>122.6949673212506</v>
       </c>
       <c r="C22" t="n">
-        <v>111.7679784405948</v>
+        <v>107.4643815002551</v>
       </c>
       <c r="D22" t="n">
-        <v>175.4165224850115</v>
+        <v>162.0129939018421</v>
       </c>
       <c r="E22" t="n">
         <v>80.87829694276101</v>
@@ -5916,13 +5916,13 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>125.9604949871992</v>
+        <v>126.086820116495</v>
       </c>
       <c r="C23" t="n">
-        <v>113.1334317282987</v>
+        <v>110.1852944249622</v>
       </c>
       <c r="D23" t="n">
-        <v>181.1419580639499</v>
+        <v>167.9689482835315</v>
       </c>
       <c r="E23" t="n">
         <v>80.36936099535117</v>
@@ -5935,13 +5935,13 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>128.097291141673</v>
+        <v>129.6086132871625</v>
       </c>
       <c r="C24" t="n">
-        <v>114.1725919301347</v>
+        <v>112.3603533751086</v>
       </c>
       <c r="D24" t="n">
-        <v>188.0009951335699</v>
+        <v>174.6552189213515</v>
       </c>
       <c r="E24" t="n">
         <v>79.75399579151699</v>
@@ -5954,13 +5954,13 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>131.4440662190809</v>
+        <v>135.4385077402319</v>
       </c>
       <c r="C25" t="n">
-        <v>116.8349325322026</v>
+        <v>117.8720468814834</v>
       </c>
       <c r="D25" t="n">
-        <v>194.2922784981469</v>
+        <v>181.7923204495455</v>
       </c>
       <c r="E25" t="n">
         <v>80.37680999091492</v>
@@ -5973,13 +5973,13 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>136.1309773416151</v>
+        <v>143.2931461814154</v>
       </c>
       <c r="C26" t="n">
-        <v>119.8466399274315</v>
+        <v>122.9567979611744</v>
       </c>
       <c r="D26" t="n">
-        <v>206.1861953857602</v>
+        <v>195.4086282085584</v>
       </c>
       <c r="E26" t="n">
         <v>81.18090769527777</v>
@@ -5992,13 +5992,13 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>140.0609263952016</v>
+        <v>147.4244111907817</v>
       </c>
       <c r="C27" t="n">
-        <v>123.6570430557842</v>
+        <v>127.4485025854801</v>
       </c>
       <c r="D27" t="n">
-        <v>210.6303430901159</v>
+        <v>198.9342324493411</v>
       </c>
       <c r="E27" t="n">
         <v>82.82088037488425</v>
@@ -6011,13 +6011,13 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>144.9088277662518</v>
+        <v>152.2273900133602</v>
       </c>
       <c r="C28" t="n">
-        <v>127.8754331719986</v>
+        <v>131.8897164220905</v>
       </c>
       <c r="D28" t="n">
-        <v>218.1864142570606</v>
+        <v>204.8842113511737</v>
       </c>
       <c r="E28" t="n">
         <v>83.94164904105426</v>
@@ -6030,13 +6030,13 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>149.7006471223579</v>
+        <v>157.1448761998557</v>
       </c>
       <c r="C29" t="n">
-        <v>132.5301178921778</v>
+        <v>136.4300084095772</v>
       </c>
       <c r="D29" t="n">
-        <v>223.5680774528964</v>
+        <v>210.105085871709</v>
       </c>
       <c r="E29" t="n">
         <v>85.60926267760219</v>
@@ -6049,13 +6049,13 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>157.3558598819894</v>
+        <v>166.5138222271086</v>
       </c>
       <c r="C30" t="n">
-        <v>138.9963995702695</v>
+        <v>144.6370989631911</v>
       </c>
       <c r="D30" t="n">
-        <v>236.3381401219637</v>
+        <v>222.2668806818258</v>
       </c>
       <c r="E30" t="n">
         <v>86.06372611542771</v>
@@ -6068,13 +6068,13 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>164.1425431061003</v>
+        <v>176.1980539327075</v>
       </c>
       <c r="C31" t="n">
-        <v>145.161794406534</v>
+        <v>154.5458575361416</v>
       </c>
       <c r="D31" t="n">
-        <v>245.7975581495947</v>
+        <v>233.197261546269</v>
       </c>
       <c r="E31" t="n">
         <v>87.69557738496161</v>

</xml_diff>

<commit_message>
Weight Riftbound singles 50:50 collector vs playable
Catalog now stores card rarity; Riftbound's singles index uses weighted
quantiles with Showcase (collector) and Common/Uncommon/Rare/Epic
(playable) buckets each carrying half the weight. Promos excluded.
Config-driven via tcg_config.RARITY_BALANCE.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GzVZ7jTqTdEEWEf8Dpoz9q
</commit_message>
<xml_diff>
--- a/output/tcg_price_trends.xlsx
+++ b/output/tcg_price_trends.xlsx
@@ -21,7 +21,6 @@
     <sheet name="DBS Fusion World" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="Sorcery" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="Weiss Schwarz" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Market composite" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -593,6 +592,10 @@
       <c r="K2" t="n">
         <v>100</v>
       </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
       <c r="P2" t="n">
         <v>100</v>
       </c>
@@ -605,6 +608,8 @@
       <c r="S2" t="n">
         <v>100</v>
       </c>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
       <c r="V2" t="n">
         <v>100</v>
       </c>
@@ -654,6 +659,10 @@
       <c r="K3" t="n">
         <v>94.16767257388445</v>
       </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
       <c r="P3" t="n">
         <v>100</v>
       </c>
@@ -721,6 +730,8 @@
       <c r="K4" t="n">
         <v>93.12695382431758</v>
       </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
       <c r="N4" t="n">
         <v>100</v>
       </c>
@@ -794,6 +805,8 @@
       <c r="K5" t="n">
         <v>94.11321988028493</v>
       </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
       <c r="N5" t="n">
         <v>109.4494720965309</v>
       </c>
@@ -867,6 +880,8 @@
       <c r="K6" t="n">
         <v>92.21201820949602</v>
       </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
       <c r="N6" t="n">
         <v>110</v>
       </c>
@@ -940,6 +955,8 @@
       <c r="K7" t="n">
         <v>92.861213452351</v>
       </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
       <c r="N7" t="n">
         <v>100.9128716988979</v>
       </c>
@@ -1013,6 +1030,8 @@
       <c r="K8" t="n">
         <v>95.52169692205069</v>
       </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
       <c r="N8" t="n">
         <v>100</v>
       </c>
@@ -1086,6 +1105,8 @@
       <c r="K9" t="n">
         <v>95.16702996950639</v>
       </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
       <c r="N9" t="n">
         <v>93.44086021505376</v>
       </c>
@@ -1159,6 +1180,8 @@
       <c r="K10" t="n">
         <v>100.948887044047</v>
       </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
       <c r="N10" t="n">
         <v>90.64054547200614</v>
       </c>
@@ -1232,6 +1255,8 @@
       <c r="K11" t="n">
         <v>103.4233299268076</v>
       </c>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
       <c r="N11" t="n">
         <v>85.71428571428569</v>
       </c>
@@ -1305,6 +1330,8 @@
       <c r="K12" t="n">
         <v>96.36645270065929</v>
       </c>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
       <c r="N12" t="n">
         <v>80</v>
       </c>
@@ -1378,6 +1405,8 @@
       <c r="K13" t="n">
         <v>96.95481310960221</v>
       </c>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
       <c r="N13" t="n">
         <v>72.14355657391953</v>
       </c>
@@ -1451,6 +1480,8 @@
       <c r="K14" t="n">
         <v>95.62160090418746</v>
       </c>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
       <c r="N14" t="n">
         <v>66.66666666666666</v>
       </c>
@@ -1524,6 +1555,8 @@
       <c r="K15" t="n">
         <v>100.6575387331966</v>
       </c>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
       <c r="N15" t="n">
         <v>62.84749034749035</v>
       </c>
@@ -1597,6 +1630,8 @@
       <c r="K16" t="n">
         <v>99.18212487945951</v>
       </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
       <c r="N16" t="n">
         <v>60.46987114500755</v>
       </c>
@@ -1670,6 +1705,8 @@
       <c r="K17" t="n">
         <v>93.76424737291555</v>
       </c>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
       <c r="N17" t="n">
         <v>60</v>
       </c>
@@ -1743,6 +1780,8 @@
       <c r="K18" t="n">
         <v>94.28552420460662</v>
       </c>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
       <c r="N18" t="n">
         <v>60.87102421943391</v>
       </c>
@@ -1816,6 +1855,8 @@
       <c r="K19" t="n">
         <v>90.54868775437416</v>
       </c>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
       <c r="N19" t="n">
         <v>61.27760557923285</v>
       </c>
@@ -1889,6 +1930,8 @@
       <c r="K20" t="n">
         <v>90.58647939902743</v>
       </c>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
       <c r="N20" t="n">
         <v>61.04336043360433</v>
       </c>
@@ -1962,6 +2005,8 @@
       <c r="K21" t="n">
         <v>87.50494337967029</v>
       </c>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
       <c r="N21" t="n">
         <v>59.2203375942314</v>
       </c>
@@ -2035,6 +2080,8 @@
       <c r="K22" t="n">
         <v>93.70820881996548</v>
       </c>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
       <c r="N22" t="n">
         <v>58.33333333333334</v>
       </c>
@@ -2188,7 +2235,7 @@
         <v>86.74178704749356</v>
       </c>
       <c r="L24" t="n">
-        <v>66.66666666666667</v>
+        <v>78.41360999845068</v>
       </c>
       <c r="M24" t="n">
         <v>128.6202013480849</v>
@@ -2267,7 +2314,7 @@
         <v>82.27970655906952</v>
       </c>
       <c r="L25" t="n">
-        <v>60.71428571428572</v>
+        <v>67.56482451545345</v>
       </c>
       <c r="M25" t="n">
         <v>130.066203922153</v>
@@ -2346,7 +2393,7 @@
         <v>82.04136295158966</v>
       </c>
       <c r="L26" t="n">
-        <v>44.44444444444445</v>
+        <v>50.35199046247254</v>
       </c>
       <c r="M26" t="n">
         <v>109.5587644735276</v>
@@ -2425,7 +2472,7 @@
         <v>85.15030441182104</v>
       </c>
       <c r="L27" t="n">
-        <v>49.63636363636363</v>
+        <v>53.66636537681402</v>
       </c>
       <c r="M27" t="n">
         <v>95.96383003098043</v>
@@ -2504,7 +2551,7 @@
         <v>86.56676038065757</v>
       </c>
       <c r="L28" t="n">
-        <v>58.53658536585365</v>
+        <v>61.27658918308845</v>
       </c>
       <c r="M28" t="n">
         <v>107.7163527937681</v>
@@ -2583,7 +2630,7 @@
         <v>88.78670617598422</v>
       </c>
       <c r="L29" t="n">
-        <v>59.45945945945946</v>
+        <v>60.26819222093938</v>
       </c>
       <c r="M29" t="n">
         <v>106.6968388573297</v>
@@ -2662,7 +2709,7 @@
         <v>87.45185443863559</v>
       </c>
       <c r="L30" t="n">
-        <v>50</v>
+        <v>44.77503895111304</v>
       </c>
       <c r="M30" t="n">
         <v>84.56221727400458</v>
@@ -2741,7 +2788,7 @@
         <v>81.27790526070994</v>
       </c>
       <c r="L31" t="n">
-        <v>46.34146341463415</v>
+        <v>41.78194993412406</v>
       </c>
       <c r="M31" t="n">
         <v>93.42062491235026</v>
@@ -7712,617 +7759,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E31"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>month</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>market_gmv_weighted</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>singles_gmv_weighted</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>sealed_gmv_weighted</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>equal_weight_typical_game</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2024-02</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>100</v>
-      </c>
-      <c r="C2" t="n">
-        <v>100</v>
-      </c>
-      <c r="D2" t="n">
-        <v>100</v>
-      </c>
-      <c r="E2" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2024-03</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>99.17439272093857</v>
-      </c>
-      <c r="C3" t="n">
-        <v>98.68861232343686</v>
-      </c>
-      <c r="D3" t="n">
-        <v>100.0577424665972</v>
-      </c>
-      <c r="E3" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2024-04</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>99.13015491220953</v>
-      </c>
-      <c r="C4" t="n">
-        <v>97.82321891205009</v>
-      </c>
-      <c r="D4" t="n">
-        <v>101.4207811604626</v>
-      </c>
-      <c r="E4" t="n">
-        <v>93.76774227364118</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2024-05</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>100.2407406378585</v>
-      </c>
-      <c r="C5" t="n">
-        <v>98.96357083695018</v>
-      </c>
-      <c r="D5" t="n">
-        <v>102.5268158994653</v>
-      </c>
-      <c r="E5" t="n">
-        <v>91.6178521859338</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2024-06</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>99.9665432915572</v>
-      </c>
-      <c r="C6" t="n">
-        <v>98.30270293736173</v>
-      </c>
-      <c r="D6" t="n">
-        <v>103.6585186698684</v>
-      </c>
-      <c r="E6" t="n">
-        <v>88.38198847677447</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2024-07</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>99.15044331481094</v>
-      </c>
-      <c r="C7" t="n">
-        <v>97.42134359130553</v>
-      </c>
-      <c r="D7" t="n">
-        <v>103.2900884310257</v>
-      </c>
-      <c r="E7" t="n">
-        <v>85.7241163578765</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2024-08</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>96.68116851514675</v>
-      </c>
-      <c r="C8" t="n">
-        <v>94.82025566188101</v>
-      </c>
-      <c r="D8" t="n">
-        <v>101.6466173469021</v>
-      </c>
-      <c r="E8" t="n">
-        <v>83.6510153432466</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2024-09</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>96.10045154310831</v>
-      </c>
-      <c r="C9" t="n">
-        <v>94.0967700879221</v>
-      </c>
-      <c r="D9" t="n">
-        <v>101.632251131286</v>
-      </c>
-      <c r="E9" t="n">
-        <v>82.69234916593996</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2024-10</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>95.49066811162173</v>
-      </c>
-      <c r="C10" t="n">
-        <v>92.56451183331282</v>
-      </c>
-      <c r="D10" t="n">
-        <v>103.1944988690451</v>
-      </c>
-      <c r="E10" t="n">
-        <v>81.65308687699158</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2024-11</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>95.54121766986984</v>
-      </c>
-      <c r="C11" t="n">
-        <v>91.83340494366114</v>
-      </c>
-      <c r="D11" t="n">
-        <v>105.2650653508497</v>
-      </c>
-      <c r="E11" t="n">
-        <v>80.17312383965516</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2024-12</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>95.69375949997942</v>
-      </c>
-      <c r="C12" t="n">
-        <v>91.25357249274218</v>
-      </c>
-      <c r="D12" t="n">
-        <v>107.3130109054414</v>
-      </c>
-      <c r="E12" t="n">
-        <v>79.55710037627702</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2025-01</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>97.15685083827383</v>
-      </c>
-      <c r="C13" t="n">
-        <v>92.1745286055498</v>
-      </c>
-      <c r="D13" t="n">
-        <v>110.1990436811134</v>
-      </c>
-      <c r="E13" t="n">
-        <v>79.03361627973339</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2025-02</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>99.85202734911758</v>
-      </c>
-      <c r="C14" t="n">
-        <v>94.07756523387819</v>
-      </c>
-      <c r="D14" t="n">
-        <v>115.3276068674647</v>
-      </c>
-      <c r="E14" t="n">
-        <v>79.15123612149803</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2025-03</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>102.5855036379036</v>
-      </c>
-      <c r="C15" t="n">
-        <v>96.55972901151149</v>
-      </c>
-      <c r="D15" t="n">
-        <v>118.8027704854365</v>
-      </c>
-      <c r="E15" t="n">
-        <v>79.83221112422456</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>2025-04</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>105.7932559796551</v>
-      </c>
-      <c r="C16" t="n">
-        <v>98.90108860664984</v>
-      </c>
-      <c r="D16" t="n">
-        <v>123.8829161231265</v>
-      </c>
-      <c r="E16" t="n">
-        <v>79.93831205908185</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>2025-05</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>107.6734361817494</v>
-      </c>
-      <c r="C17" t="n">
-        <v>99.81010488262073</v>
-      </c>
-      <c r="D17" t="n">
-        <v>127.6546497738228</v>
-      </c>
-      <c r="E17" t="n">
-        <v>79.32365291573286</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>2025-06</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>110.2170334349673</v>
-      </c>
-      <c r="C18" t="n">
-        <v>100.5045938803153</v>
-      </c>
-      <c r="D18" t="n">
-        <v>134.3506100060195</v>
-      </c>
-      <c r="E18" t="n">
-        <v>78.74636682447156</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>2025-07</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>111.4078579147555</v>
-      </c>
-      <c r="C19" t="n">
-        <v>100.1853927225251</v>
-      </c>
-      <c r="D19" t="n">
-        <v>139.6817121841773</v>
-      </c>
-      <c r="E19" t="n">
-        <v>78.67813718839194</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>2025-08</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>114.6658845009353</v>
-      </c>
-      <c r="C20" t="n">
-        <v>102.1819908933275</v>
-      </c>
-      <c r="D20" t="n">
-        <v>146.1253552532038</v>
-      </c>
-      <c r="E20" t="n">
-        <v>79.06140420966491</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>2025-09</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>118.2903683032758</v>
-      </c>
-      <c r="C21" t="n">
-        <v>103.8802198851831</v>
-      </c>
-      <c r="D21" t="n">
-        <v>154.7280760273166</v>
-      </c>
-      <c r="E21" t="n">
-        <v>78.8155554942265</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>2025-10</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>122.3540352363202</v>
-      </c>
-      <c r="C22" t="n">
-        <v>107.1332395359376</v>
-      </c>
-      <c r="D22" t="n">
-        <v>161.5338062275738</v>
-      </c>
-      <c r="E22" t="n">
-        <v>79.31715069957656</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>2025-11</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>125.7192243752519</v>
-      </c>
-      <c r="C23" t="n">
-        <v>109.8322842368129</v>
-      </c>
-      <c r="D23" t="n">
-        <v>167.4408340167471</v>
-      </c>
-      <c r="E23" t="n">
-        <v>78.84772279997634</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>2025-12</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>129.151817439095</v>
-      </c>
-      <c r="C24" t="n">
-        <v>111.3513471132339</v>
-      </c>
-      <c r="D24" t="n">
-        <v>176.2747421254005</v>
-      </c>
-      <c r="E24" t="n">
-        <v>75.89141925051054</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>2026-01</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>134.2513959854246</v>
-      </c>
-      <c r="C25" t="n">
-        <v>116.3396868358249</v>
-      </c>
-      <c r="D25" t="n">
-        <v>182.0434675982118</v>
-      </c>
-      <c r="E25" t="n">
-        <v>75.87447344724443</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>2026-02</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>141.7558988339657</v>
-      </c>
-      <c r="C26" t="n">
-        <v>121.0836650791243</v>
-      </c>
-      <c r="D26" t="n">
-        <v>195.5176962129382</v>
-      </c>
-      <c r="E26" t="n">
-        <v>74.66312510784216</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>2026-03</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>145.8769391378082</v>
-      </c>
-      <c r="C27" t="n">
-        <v>125.8014134355426</v>
-      </c>
-      <c r="D27" t="n">
-        <v>198.0964117173522</v>
-      </c>
-      <c r="E27" t="n">
-        <v>76.44851762461221</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>2026-04</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>150.79628026102</v>
-      </c>
-      <c r="C28" t="n">
-        <v>130.2136606497128</v>
-      </c>
-      <c r="D28" t="n">
-        <v>204.631838862801</v>
-      </c>
-      <c r="E28" t="n">
-        <v>78.4122906528619</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>2026-05</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>155.0340677073939</v>
-      </c>
-      <c r="C29" t="n">
-        <v>134.2516133763094</v>
-      </c>
-      <c r="D29" t="n">
-        <v>208.5598715539369</v>
-      </c>
-      <c r="E29" t="n">
-        <v>79.74481046922452</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>2026-06</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>162.8643566812212</v>
-      </c>
-      <c r="C30" t="n">
-        <v>141.3564673559492</v>
-      </c>
-      <c r="D30" t="n">
-        <v>217.6732154174342</v>
-      </c>
-      <c r="E30" t="n">
-        <v>78.88130443267931</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>2026-07</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>172.5827284401316</v>
-      </c>
-      <c r="C31" t="n">
-        <v>150.9625359695569</v>
-      </c>
-      <c r="D31" t="n">
-        <v>229.4478915814077</v>
-      </c>
-      <c r="E31" t="n">
-        <v>79.65743609510314</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -8581,13 +8017,13 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="D12" t="n">
-        <v>46.3</v>
+        <v>41.8</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.6868</v>
+        <v>-0.7321</v>
       </c>
     </row>
     <row r="13">
@@ -13895,7 +13331,7 @@
         <v>100</v>
       </c>
       <c r="E2" t="n">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="F2" t="n">
         <v>100</v>
@@ -13917,16 +13353,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>66.66666666666667</v>
+        <v>78.41360999845068</v>
       </c>
       <c r="C3" t="n">
-        <v>39.18128654970761</v>
+        <v>43.9703075291622</v>
       </c>
       <c r="D3" t="n">
-        <v>121.3114754098361</v>
+        <v>127.3616815334977</v>
       </c>
       <c r="E3" t="n">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="F3" t="n">
         <v>128.6202013480849</v>
@@ -13948,16 +13384,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>60.71428571428572</v>
+        <v>67.56482451545345</v>
       </c>
       <c r="C4" t="n">
-        <v>38.70967741935484</v>
+        <v>40.07107004841644</v>
       </c>
       <c r="D4" t="n">
-        <v>99.26892950391647</v>
+        <v>105.5631544936485</v>
       </c>
       <c r="E4" t="n">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="F4" t="n">
         <v>130.066203922153</v>
@@ -13979,16 +13415,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>44.44444444444445</v>
+        <v>50.35199046247254</v>
       </c>
       <c r="C5" t="n">
-        <v>26.92117005453644</v>
+        <v>28</v>
       </c>
       <c r="D5" t="n">
-        <v>78.57142857142857</v>
+        <v>91.44091013463044</v>
       </c>
       <c r="E5" t="n">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="F5" t="n">
         <v>109.5587644735276</v>
@@ -14010,16 +13446,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>49.63636363636363</v>
+        <v>53.66636537681402</v>
       </c>
       <c r="C6" t="n">
-        <v>30.17890772128061</v>
+        <v>29.61648837365079</v>
       </c>
       <c r="D6" t="n">
-        <v>83.31503841931944</v>
+        <v>93.57470459643002</v>
       </c>
       <c r="E6" t="n">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="F6" t="n">
         <v>95.96383003098043</v>
@@ -14041,16 +13477,16 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>58.53658536585365</v>
+        <v>61.27658918308845</v>
       </c>
       <c r="C7" t="n">
-        <v>34.48275862068966</v>
+        <v>35.05154639175258</v>
       </c>
       <c r="D7" t="n">
-        <v>100</v>
+        <v>98.92939541078465</v>
       </c>
       <c r="E7" t="n">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="F7" t="n">
         <v>107.7163527937681</v>
@@ -14072,16 +13508,16 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>59.45945945945946</v>
+        <v>60.26819222093938</v>
       </c>
       <c r="C8" t="n">
-        <v>36.272040302267</v>
+        <v>35.85561936013119</v>
       </c>
       <c r="D8" t="n">
-        <v>100</v>
+        <v>97.1525664470184</v>
       </c>
       <c r="E8" t="n">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="F8" t="n">
         <v>106.6968388573297</v>
@@ -14103,16 +13539,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>50</v>
+        <v>44.77503895111304</v>
       </c>
       <c r="C9" t="n">
-        <v>28.8235294117647</v>
+        <v>22.59421222078326</v>
       </c>
       <c r="D9" t="n">
-        <v>77.49999999999999</v>
+        <v>72.72482531602198</v>
       </c>
       <c r="E9" t="n">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="F9" t="n">
         <v>84.56221727400458</v>
@@ -14134,16 +13570,16 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>46.34146341463415</v>
+        <v>41.78194993412406</v>
       </c>
       <c r="C10" t="n">
-        <v>26.41509433962264</v>
+        <v>20.99924553582162</v>
       </c>
       <c r="D10" t="n">
-        <v>72.72727272727273</v>
+        <v>71.86751080345692</v>
       </c>
       <c r="E10" t="n">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="F10" t="n">
         <v>93.42062491235026</v>

</xml_diff>